<commit_message>
Chỉnh sửa mô hình tinh chỉnh
</commit_message>
<xml_diff>
--- a/ket_qua/ket_qua_modelKNeighbors.xlsx
+++ b/ket_qua/ket_qua_modelKNeighbors.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline Comparison" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion Matrix" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KFold" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline_3_Loai_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So_Sanh_Tuning" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_Matrix_Tuned" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KFold_Tuned" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,37 +484,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Best Parameters</t>
+          <t>Phiên bản Mô hình</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Test Accuracy (Sau Tuning)</t>
+          <t>Test Accuracy</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Mean KFold Accuracy</t>
+          <t>Bộ tham số</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 13, 'weights': 'distance'}</t>
+          <t>Baseline (Tham số mặc định)</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>0.7336244541484717</v>
       </c>
-      <c r="C2" t="n">
-        <v>0.7577568134171908</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mặc định</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuned (Đã tinh chỉnh)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.7336244541484717</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>{'metric': 'euclidean', 'n_neighbors': 13, 'weights': 'distance'}</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tuan09/TH07/Chỉnh sửa mô hình tinh chỉnh
</commit_message>
<xml_diff>
--- a/ket_qua/ket_qua_modelKNeighbors.xlsx
+++ b/ket_qua/ket_qua_modelKNeighbors.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline Comparison" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion Matrix" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KFold" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline_3_Loai_Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So_Sanh_Tuning" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_Matrix_Tuned" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KFold_Tuned" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,37 +484,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Best Parameters</t>
+          <t>Phiên bản Mô hình</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Test Accuracy (Sau Tuning)</t>
+          <t>Test Accuracy</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Mean KFold Accuracy</t>
+          <t>Bộ tham số</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 13, 'weights': 'distance'}</t>
+          <t>Baseline (Tham số mặc định)</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>0.7336244541484717</v>
       </c>
-      <c r="C2" t="n">
-        <v>0.7577568134171908</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mặc định</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuned (Đã tinh chỉnh)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.7336244541484717</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>{'metric': 'euclidean', 'n_neighbors': 13, 'weights': 'distance'}</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>